<commit_message>
Merge the two duplicate-looking weather-source rows in sources.xlsx
Rows 38 ("Πηγή καιρού", synthetic fallback) and 58 ("Πηγή καιρού
(τυπικό έτος)", the active csv_typical_year source) documented the
same weather.source parameter from two angles and looked like
duplicates at a glance, even though their content differed. Merged
into a single row covering both the active source and the fallback.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NsJmHNTzZq7wXZFmZdLYNB
</commit_message>
<xml_diff>
--- a/docs/sources.xlsx
+++ b/docs/sources.xlsx
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1917,32 +1917,32 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>weather.source</t>
+          <t>weather.source, weather.csv_path</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>synthetic</t>
+          <t>csv_typical_year (ενεργό) / synthetic (fallback)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>PLACEHOLDER (fallback, όχι πλέον default)</t>
+          <t>SOURCED (ενεργό) / PLACEHOLDER (fallback)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Συνθετική γεννήτρια καιρού (sine waves), κρατιέται μόνο ως fallback source — δες τη γραμμή 'Πηγή καιρού (τυπικό έτος)' για την ενεργή πηγή</t>
+          <t>Ενεργή πηγή: csv_typical_year -- πραγματικά ιστορικά δεδομένα (θερμοκρασία/υγρασία/ηλιακή ακτινοβολία), 10ετία 2015-2024, Αλεξάνδρεια Ημαθίας, μέσος όρος ανά μήνα/ημέρα/ώρα σε 'τυπικό έτος' από Open-Meteo. Αποκάλυψε ένα πραγματικό bug στον αερισμό (βλ. γραμμή 'Κατώφλι σκίασης') που το συνθετικό μοντέλο έκρυβε -- μετά τη διόρθωση: yield 150 ημερών 14.11-&gt;32.79 kg/m2, min εσωτερική θερμοκρασία 3.9C-&gt;15.6C. Fallback: synthetic -- συνθετική γεννήτρια καιρού (sine waves), κρατιέται μόνο ως fallback source, όχι πλέον default.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>docs/assumptions/weather.md — υψηλότερης αξίας μελλοντική αναβάθμιση: αλλαγή σε 'csv'</t>
+          <t>docs/papers/open-meteo-historical-weather-api.md</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>config/greenhouse_example.yaml</t>
+          <t>twin/weather.py, scripts/fetch_weather.py, config/greenhouse_example.yaml</t>
         </is>
       </c>
     </row>
@@ -2652,143 +2652,143 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Πηγή καιρού (τυπικό έτος)</t>
+          <t>Ενεργοποίηση fan-pad ψύξης</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>weather.source=csv_typical_year, weather.csv_path</t>
+          <t>climate_control.fan_pad_cooling_enabled</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>10ετία 2015-2024, Αλεξάνδρεια Ημαθίας</t>
+          <t>true (ενεργό σε αυτό το config, default false)</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>SOURCED (ενεργό)</t>
+          <t>Επιλογή config</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Πραγματικά ιστορικά δεδομένα (θερμοκρασία/υγρασία/ηλιακή ακτινοβολία) από Open-Meteo, μέσος όρος ανά μήνα/ημέρα/ώρα σε 'τυπικό έτος' — ενεργή πηγή καιρού (config/greenhouse_example.yaml). Αποκάλυψε ένα πραγματικό bug στον αερισμό (βλ. γραμμή 'Κατώφλι σκίασης') που το συνθετικό μοντέλο έκρυβε — μετά τη διόρθωση: yield 150 ημερών 14.11→32.79 kg/m², min εσωτερική θερμοκρασία 3.9°C→15.6°C.</t>
+          <t>Αρχική on/off επιλογή στο config για το αν το θερμοκήπιο διαθέτει σύστημα εξατμιστικής ψύξης fan-pad — ζητήθηκε ρητά από τον χρήστη. Ενεργοποιήθηκε στο ενεργό config μετά από δοκιμή 300 ημερών (1/3/2027, καλύπτει καλοκαίρι) που έδειξε μεγάλο όφελος: max εσωτερική θερμοκρασία 35.6°C→25.5°C, ώρες &gt;28°C 955→0, yield 76.67→92.26 kg/m². Default false στον κώδικα για νέα configs, καθώς δεν έχει επιβεβαιωθεί αν η πραγματική προσφορά (OptiClima cooling panels) αφορά fan-pad θερμοκρασιακή ψύξη ή μόνο αφύγρανση.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>papers/open-meteo-historical-weather-api.md</t>
+          <t>Επιλογή χρήστη, δεν υπάρχει βιβλιογραφική πηγή</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>twin/weather.py, scripts/fetch_weather.py</t>
+          <t>twin/params.py, twin/climate_model.py</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Ενεργοποίηση fan-pad ψύξης</t>
+          <t>Απόδοση fan-pad ψύξης</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>climate_control.fan_pad_cooling_enabled</t>
+          <t>climate_control.fan_pad_efficiency</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>true (ενεργό σε αυτό το config, default false)</t>
+          <t>0.80</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>Επιλογή config</t>
+          <t>SOURCED</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Αρχική on/off επιλογή στο config για το αν το θερμοκήπιο διαθέτει σύστημα εξατμιστικής ψύξης fan-pad — ζητήθηκε ρητά από τον χρήστη. Ενεργοποιήθηκε στο ενεργό config μετά από δοκιμή 300 ημερών (1/3/2027, καλύπτει καλοκαίρι) που έδειξε μεγάλο όφελος: max εσωτερική θερμοκρασία 35.6°C→25.5°C, ώρες &gt;28°C 955→0, yield 76.67→92.26 kg/m². Default false στον κώδικα για νέα configs, καθώς δεν έχει επιβεβαιωθεί αν η πραγματική προσφορά (OptiClima cooling panels) αφορά fan-pad θερμοκρασιακή ψύξη ή μόνο αφύγρανση.</t>
+          <t>Κλάσμα απόστασης από ξηρή εξωτερική θερμοκρασία προς τον υγρό βολβό (wet-bulb) που φτάνει ο αέρας μετά τα pads — UF/IFAS 85% για καλά συντηρημένο σύστημα, Alabama Extension 70-85%. Χρησιμοποιείται μαζί με τύπο Stull (2011) για wet-bulb. Ενεργοποιεί ταυτόχρονα ψύξη ΚΑΙ αύξηση υγρασίας (αδιαβατική διεργασία) στον ενεργό αερισμό.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Επιλογή χρήστη, δεν υπάρχει βιβλιογραφική πηγή</t>
+          <t>papers/fan-pad-evaporative-cooling.md</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>twin/params.py, twin/climate_model.py</t>
+          <t>twin/climate_model.py</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Απόδοση fan-pad ψύξης</t>
+          <t>Φωτοσύνθεση κόμης (self-shading)</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>climate_control.fan_pad_efficiency</t>
+          <t>_canopy_light_response (twin/crop_model.py)</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>k=0.75 (ίδιο με το υπάρχον)</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>SOURCED</t>
+          <t>SOURCED, bug fix</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Κλάσμα απόστασης από ξηρή εξωτερική θερμοκρασία προς τον υγρό βολβό (wet-bulb) που φτάνει ο αέρας μετά τα pads — UF/IFAS 85% για καλά συντηρημένο σύστημα, Alabama Extension 70-85%. Χρησιμοποιείται μαζί με τύπο Stull (2011) για wet-bulb. Ενεργοποιεί ταυτόχρονα ψύξη ΚΑΙ αύξηση υγρασίας (αδιαβατική διεργασία) στον ενεργό αερισμό.</t>
+          <t>Πριν: gross assimilation = ρυθμός ενός φύλλου στο πλήρες φως × LAI — σαν όλα τα φύλλα να έβλεπαν τον ίδιο ήλιο. Πραγματικά τα κατώτερα φύλλα σκιάζονται. Αυτό υπερεκτιμούσε δυσανάλογα περισσότερο το χαμηλό φως (χειμώνας) παρά το υψηλό (καλοκαίρι) — Νοέμβριος (89 W/m²) έδινε σχεδόν όσο ο Μάιος (262 W/m², 3x φως). Διορθώθηκε με ολοκλήρωμα Beer-Lambert/Michaelis-Menten (de Wit/Goudriaan τύπος). Yield 300 ημερών: 92.98→42.58 kg/m² (πιο ρεαλιστικό — κάτω από ολλανδικό όριο χωρίς τεχνητό φωτισμό, ενώ πριν ήταν στο επίπεδο ρεκόρ Ολλανδίας χωρίς καν να έχουμε τεχνητό φωτισμό).</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>papers/fan-pad-evaporative-cooling.md</t>
+          <t>papers/canopy-self-shading-photosynthesis.md</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>twin/climate_model.py</t>
+          <t>twin/crop_model.py</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>Φωτοσύνθεση κόμης (self-shading)</t>
+          <t>Αναφορά αναπνοής (high-water mark)</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>_canopy_light_response (twin/crop_model.py)</t>
+          <t>CropState.respiration_reference_g_m2 (twin/crop_model.py)</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>k=0.75 (ίδιο με το υπάρχον)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>SOURCED, bug fix</t>
+          <t>PLACEHOLDER, bug fix</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Πριν: gross assimilation = ρυθμός ενός φύλλου στο πλήρες φως × LAI — σαν όλα τα φύλλα να έβλεπαν τον ίδιο ήλιο. Πραγματικά τα κατώτερα φύλλα σκιάζονται. Αυτό υπερεκτιμούσε δυσανάλογα περισσότερο το χαμηλό φως (χειμώνας) παρά το υψηλό (καλοκαίρι) — Νοέμβριος (89 W/m²) έδινε σχεδόν όσο ο Μάιος (262 W/m², 3x φως). Διορθώθηκε με ολοκλήρωμα Beer-Lambert/Michaelis-Menten (de Wit/Goudriaan τύπος). Yield 300 ημερών: 92.98→42.58 kg/m² (πιο ρεαλιστικό — κάτω από ολλανδικό όριο χωρίς τεχνητό φωτισμό, ενώ πριν ήταν στο επίπεδο ρεκόρ Ολλανδίας χωρίς καν να έχουμε τεχνητό φωτισμό).</t>
+          <t>ΑΝΑΘΕΩΡΗΘΗΚΕ αυθημερόν: η πρώτη προσπάθεια (respiration_deficit_g_m2, "αποπλήρωσε πλήρως πριν καρπό") διόρθωσε το πρόσημο αλλά διπλομέτραγε την απώλεια -- ~480 απο ~1505 g/m2 συνολικής φωτοσύνθεσης (32%) εκτρεπόταν ΔΕΥΤΕΡΗ φορά, ενώ ήδη είχε αφαιρεθεί μία φορά από τη standing biomass. yield 150 ημερών έπεσε στα 6.21. Διορθώθηκε σωστά με respiration_reference_g_m2: τρέχον ιστορικό μέγιστο (high-water mark) της standing biomass -- η αναπνοή χρεώνεται σε αυτό, οχι στην τρέχουσα (συρρικνούμενη) τιμή, άρα μια κακή νύχτα κοστίζει ΜΙΑ φορά, όχι δύο. Αποτέλεσμα: yield 150 ημερών επέστρεψε στα 13.06 kg/m2 (κοντά στο 13.38 πριν τα δύο αυτά fixes), και το sweep νυχτερινού setpoint δείχνει σωστή κορυφή στους 16-17°C.</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>papers/canopy-self-shading-photosynthesis.md</t>
+          <t>docs/assumptions/crop-model.md</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -2800,72 +2800,35 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Αναφορά αναπνοής (high-water mark)</t>
+          <t>Ευαισθησία γονιμοποίησης στη θερμοκρασία</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>CropState.respiration_reference_g_m2 (twin/crop_model.py)</t>
+          <t>FRUIT_SET_T_MIN_C, FRUIT_SET_T_OPT_C, FRUIT_SET_T_MAX_C, _fruit_set_temp_response (twin/crop_model.py)</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>12.0 / 18.0 / 24.0 °C</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>PLACEHOLDER, bug fix</t>
+          <t>SOURCED, bug fix</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>ΑΝΑΘΕΩΡΗΘΗΚΕ αυθημερόν: η πρώτη προσπάθεια (respiration_deficit_g_m2, "αποπλήρωσε πλήρως πριν καρπό") διόρθωσε το πρόσημο αλλά διπλομέτραγε την απώλεια -- ~480 απο ~1505 g/m2 συνολικής φωτοσύνθεσης (32%) εκτρεπόταν ΔΕΥΤΕΡΗ φορά, ενώ ήδη είχε αφαιρεθεί μία φορά από τη standing biomass. yield 150 ημερών έπεσε στα 6.21. Διορθώθηκε σωστά με respiration_reference_g_m2: τρέχον ιστορικό μέγιστο (high-water mark) της standing biomass -- η αναπνοή χρεώνεται σε αυτό, οχι στην τρέχουσα (συρρικνούμενη) τιμή, άρα μια κακή νύχτα κοστίζει ΜΙΑ φορά, όχι δύο. Αποτέλεσμα: yield 150 ημερών επέστρεψε στα 13.06 kg/m2 (κοντά στο 13.38 πριν τα δύο αυτά fixes), και το sweep νυχτερινού setpoint δείχνει σωστή κορυφή στους 16-17°C.</t>
+          <t>Πραγματική βιβλιογραφία για ευαισθησία γονιμοποίησης (κάτω από 55°F ανθόπτωση, ιδανικό 60-70°F, πάνω από 75°F παρεμβολή γυρεοσωλήνα). Χρειάστηκε EMA θερμοκρασίας (12ωρο half-life) ώστε μια κρύα νύχτα να κουβαλάει ποινή στην επόμενη μέρα. Μετά τη διόρθωση του διπλομετρήματος αναπνοής (βλ. row 62), η κορυφή του sweep πλέον πέφτει στους 16-17°C -- πολύ κοντά στο βιβλιογραφικό 17-18°C, όχι πια στους 12°C.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>docs/assumptions/crop-model.md</t>
+          <t>papers/tomato-fruit-set-temperature-sensitivity.md</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
-        <is>
-          <t>twin/crop_model.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>Ευαισθησία γονιμοποίησης στη θερμοκρασία</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>FRUIT_SET_T_MIN_C, FRUIT_SET_T_OPT_C, FRUIT_SET_T_MAX_C, _fruit_set_temp_response (twin/crop_model.py)</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>12.0 / 18.0 / 24.0 °C</t>
-        </is>
-      </c>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>SOURCED, bug fix</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>Πραγματική βιβλιογραφία για ευαισθησία γονιμοποίησης (κάτω από 55°F ανθόπτωση, ιδανικό 60-70°F, πάνω από 75°F παρεμβολή γυρεοσωλήνα). Χρειάστηκε EMA θερμοκρασίας (12ωρο half-life) ώστε μια κρύα νύχτα να κουβαλάει ποινή στην επόμενη μέρα. Μετά τη διόρθωση του διπλομετρήματος αναπνοής (βλ. row 62), η κορυφή του sweep πλέον πέφτει στους 16-17°C -- πολύ κοντά στο βιβλιογραφικό 17-18°C, όχι πια στους 12°C.</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>papers/tomato-fruit-set-temperature-sensitivity.md</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="inlineStr">
         <is>
           <t>twin/crop_model.py</t>
         </is>

</xml_diff>

<commit_message>
Make variety-dependent crop traits fully configurable, add stems_per_plant
Moves the last hardcoded variety-related constants in twin/crop_model.py
(photosynthesis and fruit-set temperature thresholds, canopy light
extinction coefficient, maintenance respiration fraction) into CropParams
fields, so swapping the tomato variety later is a config change, not a
code change.

Also adds crop.stems_per_plant (1 or 2) as a real behavioral flag: it
scales effective canopy stem density in _lai() and changes the divisor
used to derive trusses-per-stem in api/main.py (renamed from
final_trusses_per_plant), matching how growers actually track truss
rate for multi-stem plants.

Documents all of the above in docs/assumptions/crop-model.md and
docs/sources.xlsx, and adds regression tests for the new validation
rules and the stems_per_plant density/fruit-set behavior.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NsJmHNTzZq7wXZFmZdLYNB
</commit_message>
<xml_diff>
--- a/docs/sources.xlsx
+++ b/docs/sources.xlsx
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3175,7 +3175,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>summary.final_trusses_per_plant, summary.avg_truss_rate_per_week</t>
+          <t>summary.final_trusses_per_stem, summary.avg_truss_rate_per_week</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Παράγεται διαιρώντας τη σωρευτική παραγωγή (final_yield_kg_m2) με (πυκνότητα x target_fruit_weight_g x fruits_per_truss) -- μετατροπή αναφοράς, όχι νέα φυσική διακριτής μέτρησης ταξιανθιών. Cross-check 2026-08-26: το 330ήμερο default config βγάζει ~0.27 τσαμπιά/εβδομάδα, πολύ χαμηλότερο από το πραγματικό εμπορικό benchmark (~1/εβδομάδα) -- ίδιο, ήδη τεκμηριωμένο yield gap (39.95 vs 65-70 kg/m²/έτος), όχι νέο πρόβλημα.</t>
+          <t>Παράγεται διαιρώντας τη σωρευτική παραγωγή (final_yield_kg_m2) με (πυκνότητα x stems_per_plant x target_fruit_weight_g x fruits_per_truss) -- μετατροπή αναφοράς, όχι νέα φυσική διακριτής μέτρησης ταξιανθιών. Cross-check 2026-08-26: το 330ήμερο default config βγάζει ~0.27 τσαμπιά/εβδομάδα, πολύ χαμηλότερο από το πραγματικό εμπορικό benchmark (~1/εβδομάδα) -- ίδιο, ήδη τεκμηριωμένο yield gap (39.95 vs 65-70 kg/m²/έτος), όχι νέο πρόβλημα.</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3201,6 +3201,191 @@
       <c r="G72" t="inlineStr">
         <is>
           <t>api/main.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Στελέχη ανά φυτό</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>crop.stems_per_plant</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>SITE-SPECIFIC</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>1 = single-stem (η βάση για τις πυκνότητες density_plants_per_m2/reference_density_plants_per_m2 αυτού του project), 2 = two-stem (ελέγχθηκε κατά την επιλογή ποικιλίας -- Belladona F1). Το μόνο πεδίο ποικιλίας που πραγματικά αλλάζει συμπεριφορά μοντέλου: το twin/crop_model.py _lai() κλιμακώνει την πυκνότητα κόμης με density_plants_per_m2 x stems_per_plant, και ο υπολογισμός ρυθμού ταξιανθιών στο api/main.py διαιρεί με την ίδια ενεργή πυκνότητα στελεχών (trusses ανά στέλεχος, όπως το μετράει πραγματικά ένας καλλιεργητής).</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Εσωτερική λογική μοντέλου</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>twin/params.py, twin/crop_model.py, api/main.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Θερμοκρασιακά όρια φωτοσύνθεσης</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>crop.photosynthesis_t_min_c / _t_opt_c / _t_max_c</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>10.0 / 27.0 / 35.0</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>SOURCED</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Μετακινήθηκαν 2026-08-26 από σταθερές module (T_MIN_C/T_OPT_C/T_MAX_C) του twin/crop_model.py σε πεδία CropParams, ώστε η θερμοκρασιακή ανοχή μιας ποικιλίας να είναι ρύθμιση config, όχι αλλαγή κώδικα. Ίδιες τιμές, καμία αλλαγή συμπεριφοράς στο default της EYRE RZ F1-class.</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Frontiers 10.3389/fpls.2017.00365; researchgate 323225604</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>twin/params.py, twin/crop_model.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Θερμοκρασιακά όρια fruit set</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>crop.fruit_set_t_min_c / _t_opt_c / _t_max_c</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>12.0 / 18.0 / 24.0</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>SOURCED</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Μετακινήθηκαν 2026-08-26 από σταθερές module (FRUIT_SET_T_MIN/OPT/MAX_C). Πολύ πιο στενή ανοχή από τη φωτοσύνθεση -- και το χαρακτηριστικό που πραγματικά διαφέρει σημαντικά μεταξύ πραγματικών ποικιλιών (π.χ. Merlice F1 "very good fruit set at high temperatures" vs. αυτό το EYRE RZ F1-class default).</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>docs/papers/tomato-fruit-set-temperature-sensitivity.md</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>twin/params.py, twin/crop_model.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Συντελεστής εξασθένησης φωτός κόμης</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>crop.canopy_light_extinction_coeff</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>SOURCED</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Μετακινήθηκε 2026-08-26 από σταθερά module (CANOPY_LIGHT_EXTINCTION_COEFF). Beer-Lambert συντελεστής (0.7-0.9 εύρος για high-wire κόμες τομάτας), διαφέρει κάπως ανάλογα με τη φυλλική συνήθεια μιας ποικιλίας.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>docs/papers/tomato-canopy-extinction-coefficient.md</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>twin/params.py, twin/crop_model.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Κλάσμα συντήρησης αναπνοής/ημέρα</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>crop.maintenance_respiration_fraction_per_day</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>0.015</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Μετακινήθηκε 2026-08-26 από σταθερά module (MAINTENANCE_RESPIRATION_FRACTION_PER_DAY), όχι ξεχωριστά τεκμηριωμένο. Η ζωτικότητα (και το φορτίο αναπνοής) ενός φυτού διαφέρει κάπως ανάλογα με την ποικιλία.</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>twin/params.py, twin/crop_model.py</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update remaining stale docs after hydroponics Level B: assumptions index and sources.xlsx audit trail
- frontend/src/api.ts: removed the stale ph_min_optimal/ph_max_optimal type
  fields (renamed to ph_optimal in the 2026-08-29 continuous-bell redesign,
  no longer used anywhere in the frontend)
- docs/assumptions/README.md: the file index and "known open gaps" section
  still described hydroponics Level B as "fully designed but not started" --
  updated to reflect it shipping across the last several commits, including
  the continuous-bell redesign
- docs/sources.xlsx: the per-parameter audit trail only covered hydroponics
  Level A (7 rows) and still said pH "doesn't feed any physics yet" -- added
  8 rows covering all the new Level B parameters (EC/pH optimal points and
  curvatures, the damped N/K/Mg/B tier, the informational tier, and the new
  marketable-yield outputs), and corrected the stale pH row
</commit_message>
<xml_diff>
--- a/docs/sources.xlsx
+++ b/docs/sources.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Οδηγός" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Παραδοχές'!$A$1:$G$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Παραδοχές'!$A$1:$G$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3523,7 +3523,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Συνήθως αναφερόμενο βέλτιστο εύρος διαθεσιμότητας θρεπτικών 5.5-6.5. Δεν τροφοδοτεί ακόμα καμία φυσική/απόδοση (Level B/C, μελλοντικό) -- μόνο εκτίθεται σαν config πεδίο.</t>
+          <t>Συνήθως αναφερόμενο βέλτιστο εύρος διαθεσιμότητας θρεπτικών 5.5-6.5. Τροφοδοτεί πλέον πραγματικά το marketable yield (Level B, 2026-08-29) μέσω συνεχούς παραβολικής καμπάνας γύρω από το βέλτιστο σημείο pH=5.5 -- δες γραμμές παρακάτω.</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3685,8 +3685,304 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>EC βέλτιστο σημείο (peak yield)</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>hydroponic.ec_optimal_ms_cm</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>3.0 mS/cm</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>SOURCED</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Μελέτη σε θερμοκηπιακή τομάτα βρήκε μέγιστο yield στα 3 dS/m -- ανεβαίνει συνεχώς μέχρι εκεί, πέφτει συνεχώς μετά. Αντικατέστησε (2026-08-29) μια αρχική flat-plateau υλοποίηση (μηδενική διαφορά σε όλο το εμπορικό εύρος 2.0-3.5 mS/cm) που ο χρήστης εντόπισε ως λανθασμένη -- η πραγματική βιβλιογραφική καμπύλη έχει ένα και μοναδικό peak, όχι flat top.</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>ResearchGate — The Effect of EC Levels of Nutrient Solution on the Growth, Yield, and Quality of Tomatoes (docs/assumptions/hydroponics.md)</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>twin/params.py, api/main.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>EC καμπυλότητα/όρια απώλειας (BER πάνω, έλλειψη κάτω)</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>hydroponic.ec_high_side_curvature_per_ms_cm2, ec_low_side_curvature_per_ms_cm2, ber_yield_loss_fraction_max, ec_deficiency_yield_loss_fraction_max</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>0.0444, 0.0375, 0.35 (35%), 0.50 (50%)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER (μηχανισμός SOURCED, μέγεθος εκτίμηση)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Συνεχής παραβολική απώλεια yield γύρω από το EC βέλτιστο σημείο -- κίνδυνος BER (Blossom End Rot, αλατότητα) πάνω από το peak, έλλειψη θρεπτικών κάτω από αυτό. Η καμπυλότητα επιλέχθηκε ώστε να διατηρεί περίπου το ίδιο μέγεθος απώλειας με μια προηγούμενη threshold-based υλοποίηση σε σημεία αναφοράς (π.χ. 10% απώλεια στα 4.5 mS/cm).</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>PMC — Saline Water Drip Irrigation BER Incidence, γενική καθοδήγηση καλλιεργητών (docs/assumptions/hydroponics.md)</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>twin/params.py, api/main.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>pH βέλτιστο σημείο (peak yield)</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>hydroponic.ph_optimal</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>SOURCED</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Πείραμα με pH 4.5/5.0/5.5/6.0/6.5 βρήκε μέγιστο yield ακριβώς στο 5.5. Αντικατέστησε (2026-08-29) μια αρχική flat-plateau υλοποίηση (5.5-6.5, μηδενική διαφορά σε όλο το εύρος) που ο χρήστης εντόπισε ως λανθασμένη -- ίδιο πρόβλημα με το EC παραπάνω.</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>ResearchGate — The Influence of pH of Nutrient Solution On Yield and Nutritional Status of Tomato Plants (docs/assumptions/hydroponics.md)</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>twin/params.py, api/main.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>pH καμπυλότητα/cap διαθεσιμότητας θρεπτικών</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>hydroponic.ph_curvature_per_ph_unit2, ph_availability_penalty_cap_fraction</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>0.0667, 0.15 (15%)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER (μηχανισμός SOURCED, μέγεθος εκτίμηση)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Συνεχής παραβολική απώλεια γύρω από το pH βέλτιστο σημείο -- κανένα ποσοτικοποιημένο ποσοστό δεν βρέθηκε στη βιβλιογραφία. Το cap είναι υψηλότερο από κάθε μεμονωμένο θρεπτικό στο damped tier παρακάτω, γιατί το pH γκαρδάρει τη διαθεσιμότητα όλων των θρεπτικών ταυτόχρονα, όχι μόνο ενός.</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>docs/assumptions/hydroponics.md</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>twin/params.py, api/main.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>N/K/Mg/B στόχοι + εύρη επάρκειας (damped tier)</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>hydroponic.n_ppm/n_min_optimal_ppm/n_max_optimal_ppm, k_*, mg_*, b_*</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>N=105 (60-150), K=300 (199-400), Mg=65 (45-70), B=0.40 (0.30-0.50) ppm</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>SOURCED εύρη, PLACEHOLDER μηχανισμός ποινής</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Εύρη από CEAC Arizona / Florida IFAS συνταγές θερμοκηπιακής τομάτας (Mg επιβεβαιώθηκε 2026-08-28 με άμεσο recheck του CEAC PDF). Πραγματικός αλλά σκόπιμα περιορισμένος (capped) μηχανισμός -- εντός εύρους καμία επίδραση στο marketable yield, εκτός γραμμική ποινή έως το ατομικό cap (βλ. επόμενη γραμμή).</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>CEAC Arizona tomato formula PDF, Florida EDIS HS796/CV216 (docs/assumptions/hydroponics.md)</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>twin/params.py, api/main.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Cap ποινής/floor damped tier</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>hydroponic.damped_nutrient_penalty_cap_fraction, recipe_adequacy_multiplier_min</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>0.02 (2% ανά θρεπτικό), 0.85 (85% floor)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>PLACEHOLDER</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Κάθε θρεπτικό (N/K/Mg/B) capped στο 2% ατομική ποινή όταν είναι ένα πλήρες εύρος-πλάτος εκτός επάρκειας· ο συνδυασμένος πολλαπλασιαστής των τεσσάρων clamped στο 0.85 ώστε το tier να μην μπορεί ποτέ να δώσει δυσανάλογα μεγάλη μεταβολή στο yield.</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>docs/assumptions/hydroponics.md</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>twin/params.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>P/S/Fe/Mn/Zn/Cu/Mo (πληροφοριακό tier)</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>hydroponic.p_ppm, s_ppm, fe_ppm, mn_ppm, zn_ppm, cu_ppm, mo_ppm</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>P=62, S=110, Fe=2.5, Mn=0.55, Zn=0.33, Cu=0.05, Mo=0.05 ppm</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>SOURCED</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>CEAC Arizona συνταγή -- μόνο εμφάνιση στο tab «Συνταγή γεωπονίας», καμία επίδραση στη φυσική (ίδια μεταχείριση με το block επικονίασης). Σημαντική απόκλιση πηγών στο Mn/Zn έναντι Florida IFAS (Zn: 0.33 vs 0.09 ppm, 3.6x διαφορά) -- τεκμηριωμένη, όχι επιλυμένη.</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>CEAC Arizona tomato formula PDF (docs/assumptions/hydroponics.md)</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>twin/params.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Marketable yield (Level B, έξοδοι)</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>summary.ec_adjusted_final_yield_kg_m2, ber_yield_loss_fraction, ec_deficiency_yield_loss_fraction, ph_availability_multiplier, recipe_adequacy_multiplier, marketable_yield_kg_m2, total_marketable_yield_kg, daily_series.marketable_yield_kg_m2</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Derived output</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Το marketable yield (μετά EC/pH/θρεπτικά) υπολογίζεται σαν σταθερός πολλαπλασιαστικός παράγοντας πάνω στο ακατέργαστο yield του crop model -- ίδιο μοτίβο reporting-layer με το Level A. Το ίδιο ratio εφαρμόζεται σε κάθε ημέρα του daily_series (2026-08-29, διόρθωση) ώστε όλες οι απεικονίσεις yield στην εφαρμογή (header, tabs, σχηματικό) να είναι συνεπείς με το marketable yield, όχι μόνο το tab «Συνταγή γεωπονίας».</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>docs/assumptions/hydroponics.md</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>twin/params.py, api/main.py</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G55"/>
+  <autoFilter ref="A1:G93"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>